<commit_message>
fixed loading and rendering of data from excel file
</commit_message>
<xml_diff>
--- a/public/data/MG_cafes.xlsx
+++ b/public/data/MG_cafes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kasia\mug-guide\public\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bastd\Documents\Git_repos\mug_guide\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{509E0B8D-225D-44C9-8186-2D4FAB7EC91D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C1F136F-BE2A-4120-89F7-84EFFA3127FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
   <si>
     <t>opinion</t>
   </si>
@@ -118,6 +118,24 @@
   </si>
   <si>
     <t>Konrad Café &amp; Bar</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>berlin</t>
+  </si>
+  <si>
+    <t>vienna</t>
+  </si>
+  <si>
+    <t>paris</t>
+  </si>
+  <si>
+    <t>warsaw</t>
+  </si>
+  <si>
+    <t>zurich</t>
   </si>
 </sst>
 </file>
@@ -170,7 +188,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,9 +197,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -465,10 +480,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -490,8 +505,11 @@
       <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="H1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -510,11 +528,14 @@
       <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="4">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G2" s="2">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -530,8 +551,11 @@
       <c r="G3">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -547,8 +571,11 @@
       <c r="G4">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -564,8 +591,11 @@
       <c r="G5">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -581,8 +611,11 @@
       <c r="G6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -598,8 +631,11 @@
       <c r="G7">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -615,8 +651,11 @@
       <c r="G8">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -632,8 +671,11 @@
       <c r="G9">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -649,8 +691,11 @@
       <c r="G10">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -666,8 +711,11 @@
       <c r="G11">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -683,8 +731,11 @@
       <c r="G12">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -700,8 +751,11 @@
       <c r="G13">
         <v>5</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -717,8 +771,11 @@
       <c r="G14">
         <v>5</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -734,8 +791,11 @@
       <c r="G15">
         <v>5</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -751,8 +811,11 @@
       <c r="G16">
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -768,8 +831,11 @@
       <c r="G17">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -785,8 +851,11 @@
       <c r="G18">
         <v>5</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -802,8 +871,11 @@
       <c r="G19">
         <v>5</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -819,8 +891,11 @@
       <c r="G20">
         <v>5</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -836,8 +911,11 @@
       <c r="G21">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -853,8 +931,11 @@
       <c r="G22">
         <v>5</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H22" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -869,6 +950,9 @@
       </c>
       <c r="G23">
         <v>5</v>
+      </c>
+      <c r="H23" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>